<commit_message>
Extend the LAMBDA test document with optional and callable cases
Add cases for the OOXML forms the import now understands: optional
parameters written with the _xlop. prefix and a built-in function passed
as a value with the _xleta. prefix, along with further callable and MAP
cases. Loading and reloading the document as XLSX then checks that these
forms survive the round-trip.

Signed-off-by: Tomaž Vajngerl <tomaz.vajngerl@collabora.co.uk>
Change-Id: I0e9acad066de12577cd40d410e25270241a406fe
Reviewed-on: https://gerrit.collaboraoffice.com/c/online/+/5784
Tested-by: Jenkins CPCI <releng@collaboraoffice.com>
Reviewed-by: Miklos Vajna <vmiklos@collabora.com>
(cherry picked from commit 6498928cf2ab2e03f8597d85717b0545d03985a9)
Reviewed-on: https://gerrit.libreoffice.org/c/core/+/207893
Tested-by: Jenkins
Reviewed-by: Xisco Fauli <xiscofauli@libreoffice.org>
</commit_message>
<xml_diff>
--- a/sc/qa/unit/data/xlsx/LambdaAndRelatedFunctions.xlsx
+++ b/sc/qa/unit/data/xlsx/LambdaAndRelatedFunctions.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30219"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{812281D3-F91B-47B8-BDF4-C25DC7FC7333}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{47FC375C-578E-4C91-9940-42CE21C19161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="3" r:id="rId1"/>
@@ -19,6 +19,8 @@
     <sheet name="Function_Scan" sheetId="9" r:id="rId9"/>
   </sheets>
   <definedNames>
+    <definedName name="APPLYTWICE">_xlfn.LAMBDA(_xlpm.f,_xlpm.x, _xlpm.f(_xlpm.f(_xlpm.x)))</definedName>
+    <definedName name="DATARANGE">Function_Lambda!$F$2:$F$5</definedName>
     <definedName name="PLUS2">_xlfn.LAMBDA(_xlpm.x, _xlpm.x+2)</definedName>
     <definedName name="SUM">_xlfn.LAMBDA(_xlpm.x,_xlpm.x+10)</definedName>
   </definedNames>
@@ -60,11 +62,18 @@
       </extLst>
     </bk>
   </futureMetadata>
-  <futureMetadata name="XLRICHVALUE" count="1">
+  <futureMetadata name="XLRICHVALUE" count="2">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
           <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="1"/>
         </ext>
       </extLst>
     </bk>
@@ -74,16 +83,19 @@
       <rc t="1" v="0"/>
     </bk>
   </cellMetadata>
-  <valueMetadata count="1">
+  <valueMetadata count="2">
     <bk>
       <rc t="2" v="0"/>
+    </bk>
+    <bk>
+      <rc t="2" v="1"/>
     </bk>
   </valueMetadata>
 </metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="83">
   <si>
     <t>LAMBDA and related Functions</t>
   </si>
@@ -139,9 +151,39 @@
     <t>COMMENT</t>
   </si>
   <si>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>Constant</t>
+  </si>
+  <si>
+    <t>Reference as input</t>
+  </si>
+  <si>
+    <t>Value as input</t>
+  </si>
+  <si>
+    <t>Unspecified value is defaulting to 0</t>
+  </si>
+  <si>
+    <t>Div by 0</t>
+  </si>
+  <si>
+    <t>Missing required parameter</t>
+  </si>
+  <si>
     <t>LAMBDA in a LET function</t>
   </si>
   <si>
+    <t>Array input</t>
+  </si>
+  <si>
+    <t>Range input</t>
+  </si>
+  <si>
+    <t>Name (of a range) input</t>
+  </si>
+  <si>
     <t>Recursive LAMBDA</t>
   </si>
   <si>
@@ -151,6 +193,99 @@
     <t>SUM LAMBDA function is set in Name Manager, make sure built-in function has priority</t>
   </si>
   <si>
+    <t>If you use SUM in LAMBDA, it will use the built-in function not the named LAMBDA</t>
+  </si>
+  <si>
+    <t>If you use SUM as parameter to LAMBDA, the named LAMBDA will be used instead</t>
+  </si>
+  <si>
+    <t>Named lambda as parameter</t>
+  </si>
+  <si>
+    <t>ETA-LAMBDA use in LAMBDA as parameter</t>
+  </si>
+  <si>
+    <t>LAMBDA as parameter to LAMBDA</t>
+  </si>
+  <si>
+    <t>Call LAMBDA 2 times</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Export of a named LAMBDA that takes a LAMBDA argument </t>
+  </si>
+  <si>
+    <t>A LAMBDA body that closes over a sheet cell</t>
+  </si>
+  <si>
+    <t>Tripple curry</t>
+  </si>
+  <si>
+    <t>Value not written - second parameter</t>
+  </si>
+  <si>
+    <t>Value not written - first parameter</t>
+  </si>
+  <si>
+    <t>TODO - Optional used but not set - number</t>
+  </si>
+  <si>
+    <t>xy</t>
+  </si>
+  <si>
+    <t>TODO - Optional used but not set - string</t>
+  </si>
+  <si>
+    <t>Syntax Error</t>
+  </si>
+  <si>
+    <t>Manual check</t>
+  </si>
+  <si>
+    <t>=LAMBDA(AX1, AX1, 0)</t>
+  </si>
+  <si>
+    <t>AX1 = cell reference name - invalid syntax</t>
+  </si>
+  <si>
+    <t>=LAMBDA([x], y, 0)</t>
+  </si>
+  <si>
+    <t>Optional, then required parameter - invalid syntax</t>
+  </si>
+  <si>
+    <t>=LAMBDA(x$, 0)</t>
+  </si>
+  <si>
+    <t>=LAMBDA(ab!, 0)</t>
+  </si>
+  <si>
+    <t>=LAMBDA(aa#a, 0)</t>
+  </si>
+  <si>
+    <t>=LAMBDA(a%, 0)</t>
+  </si>
+  <si>
+    <t>=LAMBDA(xx@3, 0)</t>
+  </si>
+  <si>
+    <t>=LAMBDA(x,y,z, {x,y,z}))(1,2,3)</t>
+  </si>
+  <si>
+    <t>Can't create an array from parameters</t>
+  </si>
+  <si>
+    <t>=LAMBDA("x", 0)(1)</t>
+  </si>
+  <si>
+    <t>TODO - Optional parameter, set</t>
+  </si>
+  <si>
+    <t>TODO - Optional parameter, not set</t>
+  </si>
+  <si>
+    <t>TODO - Required parameter, not set</t>
+  </si>
+  <si>
     <t>ABC</t>
   </si>
   <si>
@@ -163,9 +298,15 @@
     <t>CF</t>
   </si>
   <si>
+    <t>Column reduction over a real range</t>
+  </si>
+  <si>
     <t>DEF</t>
   </si>
   <si>
+    <t>Row reduction over a real range</t>
+  </si>
+  <si>
     <t>DATA</t>
   </si>
   <si>
@@ -175,14 +316,41 @@
     <t>B</t>
   </si>
   <si>
+    <t>Element map over a range</t>
+  </si>
+  <si>
+    <t>Data 1</t>
+  </si>
+  <si>
+    <t>Data 2</t>
+  </si>
+  <si>
     <t>abc</t>
+  </si>
+  <si>
+    <t>10_abc</t>
+  </si>
+  <si>
+    <t>REDUCE over a 2D array</t>
+  </si>
+  <si>
+    <t>REDUCE over a range</t>
+  </si>
+  <si>
+    <t>aa</t>
+  </si>
+  <si>
+    <t>aab</t>
+  </si>
+  <si>
+    <t>aabc</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -207,6 +375,14 @@
       <b/>
       <sz val="28"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -238,7 +414,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -256,11 +432,70 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="10">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color theme="1"/>
@@ -335,9 +570,14 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="2">
   <rv s="0">
     <v>2</v>
+    <v>2</v>
+    <v>19</v>
+  </rv>
+  <rv s="0">
+    <v>1</v>
     <v>2</v>
     <v>19</v>
   </rv>
@@ -695,7 +935,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="b">
-        <f>AND(Function_Lambda!C2:C100)</f>
+        <f>AND(Function_Lambda!C2:C107)</f>
         <v>1</v>
       </c>
     </row>
@@ -749,7 +989,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="5" t="b">
-        <f>AND(Function_Reduce!C2:C100)</f>
+        <f>AND(Function_Reduce!C2:C102)</f>
         <v>1</v>
       </c>
     </row>
@@ -767,12 +1007,12 @@
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <conditionalFormatting sqref="B3">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="2" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:B13">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
@@ -782,17 +1022,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="2" max="2" width="15.5703125" customWidth="1"/>
     <col min="3" max="3" width="23.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="91.140625" customWidth="1"/>
     <col min="5" max="5" width="85.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="A1" s="4" t="s">
         <v>13</v>
       </c>
@@ -808,8 +1048,11 @@
       <c r="E1" s="4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="F1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2" cm="1">
         <f t="array" ref="A2">_xlfn.LAMBDA(_xlpm.a, 2)(1)</f>
         <v>2</v>
@@ -825,403 +1068,862 @@
         <f ca="1">_xlfn.FORMULATEXT(A2)</f>
         <v>=LAMBDA(a, 2)(1)</v>
       </c>
-    </row>
-    <row r="3" spans="1:5">
+      <c r="E2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" cm="1">
-        <f t="array" ref="A3">_xlfn.LAMBDA(_xlpm.a, _xlpm.a)(3)</f>
-        <v>3</v>
+        <f t="array" ref="A3">_xlfn.LAMBDA(_xlpm.a, _xlpm.a)(F2)</f>
+        <v>10</v>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="C3" s="2" t="b">
         <f>A3=B3</f>
         <v>1</v>
       </c>
       <c r="D3" s="1" t="str">
-        <f t="shared" ref="D3:D24" ca="1" si="0">_xlfn.FORMULATEXT(A3)</f>
-        <v>=LAMBDA(a, a)(3)</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
+        <f ca="1">_xlfn.FORMULATEXT(A3)</f>
+        <v>=LAMBDA(a, a)(F2)</v>
+      </c>
+      <c r="E3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4" cm="1">
-        <f t="array" ref="A4">_xlfn.LAMBDA(_xlpm.a, _xlpm.a * 2)(2)</f>
-        <v>4</v>
+        <f t="array" ref="A4">_xlfn.LAMBDA(_xlpm.a, _xlpm.a)(3)</f>
+        <v>3</v>
       </c>
       <c r="B4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C4" s="2" t="b">
         <f>A4=B4</f>
         <v>1</v>
       </c>
       <c r="D4" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
+        <f ca="1">_xlfn.FORMULATEXT(A4)</f>
+        <v>=LAMBDA(a, a)(3)</v>
+      </c>
+      <c r="E4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" cm="1">
+        <f t="array" ref="A5">_xlfn.LAMBDA(_xlpm.a, _xlpm.a * 2)(2)</f>
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2" t="b">
+        <f>A5=B5</f>
+        <v>1</v>
+      </c>
+      <c r="D5" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A5)</f>
         <v>=LAMBDA(a, a * 2)(2)</v>
       </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" cm="1">
-        <f t="array" ref="A5">_xlfn.LAMBDA(_xlpm.x,_xlpm.y, _xlpm.x + _xlpm.y)(3, 4)</f>
+      <c r="F5">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" cm="1">
+        <f t="array" ref="A6">_xlfn.LAMBDA(_xlpm.x,_xlpm.y, _xlpm.x + _xlpm.y)(3, 4)</f>
         <v>7</v>
       </c>
-      <c r="B5">
+      <c r="B6">
         <v>7</v>
       </c>
-      <c r="C5" s="2" t="b">
-        <f t="shared" ref="C5:C24" si="1">A5=B5</f>
-        <v>1</v>
-      </c>
-      <c r="D5" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="C6" s="2" t="b">
+        <f>A6=B6</f>
+        <v>1</v>
+      </c>
+      <c r="D6" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A6)</f>
         <v>=LAMBDA(x,y, x + y)(3, 4)</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
-      <c r="A6" cm="1">
-        <f t="array" ref="A6">_xlfn.LAMBDA(_xlpm.a, _xlpm.a+_xlpm.a)(5)</f>
+    <row r="7" spans="1:6">
+      <c r="A7" cm="1">
+        <f t="array" ref="A7">_xlfn.LAMBDA(_xlpm.a, _xlpm.a + _xlpm.a)(5)</f>
         <v>10</v>
       </c>
-      <c r="B6">
+      <c r="B7">
         <v>10</v>
       </c>
-      <c r="C6" s="2" t="b">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="D6" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>=LAMBDA(a, a+a)(5)</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" cm="1">
-        <f t="array" ref="A7">_xlfn.LAMBDA(_xlpm.x,_xlpm.y, _xlpm.x * _xlpm.y + _xlpm.x)(3, 4)</f>
+      <c r="C7" s="2" t="b">
+        <f>A7=B7</f>
+        <v>1</v>
+      </c>
+      <c r="D7" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A7)</f>
+        <v>=LAMBDA(a, a + a)(5)</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" cm="1">
+        <f t="array" ref="A8">_xlfn.LAMBDA(_xlpm.x,_xlpm.y, _xlpm.x * _xlpm.y + _xlpm.x)(3, 4)</f>
         <v>15</v>
       </c>
-      <c r="B7">
+      <c r="B8">
         <v>15</v>
       </c>
-      <c r="C7" s="2" t="b">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="D7" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="C8" s="2" t="b">
+        <f>A8=B8</f>
+        <v>1</v>
+      </c>
+      <c r="D8" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A8)</f>
         <v>=LAMBDA(x,y, x * y + x)(3, 4)</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
-      <c r="A8" cm="1">
-        <f t="array" ref="A8">_xlfn.LAMBDA(_xlpm.a, IF(_xlpm.a &gt; 0, _xlpm.a, -_xlpm.a))(-5)</f>
+    <row r="9" spans="1:6">
+      <c r="A9" cm="1">
+        <f t="array" ref="A9">_xlfn.LAMBDA(_xlpm.a, IF(_xlpm.a &gt; 0, _xlpm.a, -_xlpm.a))(-5)</f>
         <v>5</v>
       </c>
-      <c r="B8">
+      <c r="B9">
         <v>5</v>
       </c>
-      <c r="C8" s="2" t="b">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="D8" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="C9" s="2" t="b">
+        <f>A9=B9</f>
+        <v>1</v>
+      </c>
+      <c r="D9" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A9)</f>
         <v>=LAMBDA(a, IF(a &gt; 0, a, -a))(-5)</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
-      <c r="A9" t="str" cm="1">
-        <f t="array" ref="A9">_xlfn.LAMBDA(_xlpm.a, _xlpm.a &amp; "!")("hi")</f>
+    <row r="10" spans="1:6">
+      <c r="A10" t="str" cm="1">
+        <f t="array" ref="A10">_xlfn.LAMBDA(_xlpm.a, _xlpm.a &amp; "!")("hi")</f>
         <v>hi!</v>
       </c>
-      <c r="B9" t="str" cm="1">
-        <f t="array" ref="B9">_xlfn.LAMBDA(_xlpm.a, _xlpm.a &amp; "!")("hi")</f>
+      <c r="B10" t="str" cm="1">
+        <f t="array" ref="B10">_xlfn.LAMBDA(_xlpm.a, _xlpm.a &amp; "!")("hi")</f>
         <v>hi!</v>
       </c>
-      <c r="C9" s="2" t="b">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="D9" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="C10" s="2" t="b">
+        <f>A10=B10</f>
+        <v>1</v>
+      </c>
+      <c r="D10" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A10)</f>
         <v>=LAMBDA(a, a &amp; "!")("hi")</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
-      <c r="A10" cm="1">
-        <f t="array" ref="A10">_xlfn.LAMBDA(_xlpm.SQRT, SQRT(_xlpm.SQRT))(4)</f>
+    <row r="11" spans="1:6">
+      <c r="A11" cm="1">
+        <f t="array" ref="A11">_xlfn.LAMBDA(_xlpm.SQRT, SQRT(_xlpm.SQRT))(4)</f>
         <v>2</v>
       </c>
-      <c r="B10">
+      <c r="B11">
         <v>2</v>
       </c>
-      <c r="C10" s="2" t="b">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="D10" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="C11" s="2" t="b">
+        <f>A11=B11</f>
+        <v>1</v>
+      </c>
+      <c r="D11" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A11)</f>
         <v>=LAMBDA(SQRT, SQRT(SQRT))(4)</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
-      <c r="A11" cm="1">
-        <f t="array" ref="A11">_xlfn.LAMBDA(_xlpm.r, SUM(_xlpm.r))(A1:A3)</f>
-        <v>5</v>
-      </c>
-      <c r="B11">
-        <v>5</v>
-      </c>
-      <c r="C11" s="2" t="b">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="D11" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>=LAMBDA(r, SUM(r))(A1:A3)</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:6">
       <c r="A12" cm="1">
-        <f t="array" ref="A12">_xlfn.LAMBDA(_xlpm.a,_xlpm.b,_xlpm.c, _xlpm.a + _xlpm.b + _xlpm.c)(1, 2, 3)</f>
+        <f t="array" ref="A12">_xlfn.LAMBDA(_xlpm.r, SUM(_xlpm.r))(F2:F5)</f>
+        <v>100</v>
+      </c>
+      <c r="B12">
+        <v>100</v>
+      </c>
+      <c r="C12" s="2" t="b">
+        <f>A12=B12</f>
+        <v>1</v>
+      </c>
+      <c r="D12" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A12)</f>
+        <v>=LAMBDA(r, SUM(r))(F2:F5)</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" cm="1">
+        <f t="array" ref="A13">_xlfn.LAMBDA(_xlpm.a,_xlpm.b,_xlpm.c, _xlpm.a + _xlpm.b + _xlpm.c)(1, 2, 3)</f>
         <v>6</v>
       </c>
-      <c r="B12">
+      <c r="B13">
         <v>6</v>
       </c>
-      <c r="C12" s="2" t="b">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="D12" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="C13" s="2" t="b">
+        <f>A13=B13</f>
+        <v>1</v>
+      </c>
+      <c r="D13" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A13)</f>
         <v>=LAMBDA(a,b,c, a + b + c)(1, 2, 3)</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
-      <c r="A13" t="b" cm="1">
-        <f t="array" ref="A13">_xlfn.LAMBDA(_xlpm.x, _xlpm.x &gt; 5)(7)</f>
-        <v>1</v>
-      </c>
-      <c r="B13" t="b">
-        <v>1</v>
-      </c>
-      <c r="C13" s="2" t="b">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="D13" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
+    <row r="14" spans="1:6">
+      <c r="A14" cm="1">
+        <f t="array" ref="A14">_xlfn.LAMBDA(_xlpm.a,_xlpm.b,_xlpm.c, _xlpm.a + _xlpm.b + _xlpm.c)(,,)</f>
+        <v>0</v>
+      </c>
+      <c r="B14">
+        <v>0</v>
+      </c>
+      <c r="C14" s="2" t="b">
+        <f>A14=B14</f>
+        <v>1</v>
+      </c>
+      <c r="D14" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A14)</f>
+        <v>=LAMBDA(a,b,c, a + b + c)(,,)</v>
+      </c>
+      <c r="E14" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" t="b" cm="1">
+        <f t="array" ref="A15">_xlfn.LAMBDA(_xlpm.x, _xlpm.x &gt; 5)(7)</f>
+        <v>1</v>
+      </c>
+      <c r="B15" t="b">
+        <v>1</v>
+      </c>
+      <c r="C15" s="2" t="b">
+        <f>A15=B15</f>
+        <v>1</v>
+      </c>
+      <c r="D15" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A15)</f>
         <v>=LAMBDA(x, x &gt; 5)(7)</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
-      <c r="A14" t="e" cm="1">
-        <f t="array" ref="A14">_xlfn.LAMBDA(_xlpm.x, 1 / _xlpm.x)(0)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="B14" t="e">
-        <v>#DIV/0!</v>
-      </c>
-      <c r="C14" s="2" t="b">
-        <f>IF(ERROR.TYPE(A14) = 2, TRUE, FALSE)</f>
-        <v>1</v>
-      </c>
-      <c r="D14" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>=LAMBDA(x, 1 / x)(0)</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5">
-      <c r="A15" t="e" cm="1" vm="1">
-        <f t="array" ref="A15">_xlfn.LAMBDA(_xlpm.x,_xlpm.y, _xlpm.x + _xlpm.y)(1)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="B15" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C15" s="2" t="b">
-        <f>IF(ERROR.TYPE(A15) = 3, TRUE, FALSE)</f>
-        <v>1</v>
-      </c>
-      <c r="D15" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>=LAMBDA(x,y, x + y)(1)</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:6">
       <c r="A16" cm="1">
-        <f t="array" ref="A16">_xlfn.LAMBDA(_xlpm.x, _xlfn.LAMBDA(_xlpm.y, _xlpm.x + _xlpm.y))(3)(4)</f>
-        <v>7</v>
+        <f t="array" ref="A16">ERROR.TYPE(_xlfn.LAMBDA(_xlpm.x, 1 / _xlpm.x)(0))</f>
+        <v>2</v>
       </c>
       <c r="B16">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C16" s="2" t="b">
-        <f t="shared" si="1"/>
+        <f>A16=B16</f>
         <v>1</v>
       </c>
       <c r="D16" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>=LAMBDA(x, LAMBDA(y, x + y))(3)(4)</v>
+        <f ca="1">_xlfn.FORMULATEXT(A16)</f>
+        <v>=ERROR.TYPE(LAMBDA(x, 1 / x)(0))</v>
+      </c>
+      <c r="E16" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" cm="1">
-        <f t="array" ref="A17">_xlfn.LET(_xlpm.f, _xlfn.LAMBDA(_xlpm.x, _xlpm.x * _xlpm.x), _xlpm.f(4))</f>
-        <v>16</v>
+        <f t="array" ref="A17">ERROR.TYPE(_xlfn.LAMBDA(_xlpm.x,_xlpm.y, _xlpm.x + _xlpm.y)(1))</f>
+        <v>3</v>
       </c>
       <c r="B17">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="C17" s="2" t="b">
-        <f t="shared" si="1"/>
+        <f>A17=B17</f>
         <v>1</v>
       </c>
       <c r="D17" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>=LET(f, LAMBDA(x, x * x), f(4))</v>
+        <f ca="1">_xlfn.FORMULATEXT(A17)</f>
+        <v>=ERROR.TYPE(LAMBDA(x,y, x + y)(1))</v>
       </c>
       <c r="E17" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" cm="1">
-        <f t="array" ref="A18">_xlfn.LAMBDA(_xlpm.a, SUM(_xlpm.a))({1;2;3})</f>
-        <v>6</v>
+        <f t="array" ref="A18">_xlfn.LAMBDA(_xlpm.x, _xlfn.LAMBDA(_xlpm.y, _xlpm.x + _xlpm.y))(3)(4)</f>
+        <v>7</v>
       </c>
       <c r="B18">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C18" s="2" t="b">
-        <f t="shared" si="1"/>
+        <f>A18=B18</f>
         <v>1</v>
       </c>
       <c r="D18" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>=LAMBDA(a, SUM(a))({1;2;3})</v>
+        <f ca="1">_xlfn.FORMULATEXT(A18)</f>
+        <v>=LAMBDA(x, LAMBDA(y, x + y))(3)(4)</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" cm="1">
-        <f t="array" ref="A19:A21">_xlfn.LAMBDA(_xlpm.a, _xlpm.a * 2)({1;2;3})</f>
-        <v>2</v>
+        <f t="array" ref="A19">_xlfn.LET(_xlpm.f, _xlfn.LAMBDA(_xlpm.x, _xlpm.x * _xlpm.x), _xlpm.f(4))</f>
+        <v>16</v>
       </c>
       <c r="B19">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="C19" s="2" t="b">
-        <f t="shared" si="1"/>
+        <f>A19=B19</f>
         <v>1</v>
       </c>
       <c r="D19" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>=LAMBDA(a, a * 2)({1;2;3})</v>
+        <f ca="1">_xlfn.FORMULATEXT(A19)</f>
+        <v>=LET(f, LAMBDA(x, x * x), f(4))</v>
+      </c>
+      <c r="E19" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20">
-        <v>4</v>
+      <c r="A20" cm="1">
+        <f t="array" ref="A20">_xlfn.LAMBDA(_xlpm.a, SUM(_xlpm.a))({1;2;3})</f>
+        <v>6</v>
       </c>
       <c r="B20">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C20" s="2" t="b">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="D20" s="1"/>
+        <f>A20=B20</f>
+        <v>1</v>
+      </c>
+      <c r="D20" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A20)</f>
+        <v>=LAMBDA(a, SUM(a))({1;2;3})</v>
+      </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21">
-        <v>6</v>
+      <c r="A21" cm="1">
+        <f t="array" ref="A21">SUM(_xlfn.LAMBDA(_xlpm.a, _xlpm.a * 2)({10;11;20}))</f>
+        <v>82</v>
       </c>
       <c r="B21">
-        <v>6</v>
+        <v>82</v>
       </c>
       <c r="C21" s="2" t="b">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="D21" s="1"/>
+        <f>A21=B21</f>
+        <v>1</v>
+      </c>
+      <c r="D21" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A21)</f>
+        <v>=SUM(LAMBDA(a, a * 2)({10;11;20}))</v>
+      </c>
+      <c r="E21" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" cm="1">
-        <f t="array" ref="A22">_xlfn.LET(_xlpm.g, _xlfn.LAMBDA(_xlpm.self,_xlpm.n, IF(_xlpm.n &lt;= 1, 1, _xlpm.n * _xlpm.self(_xlpm.self, _xlpm.n - 1))), _xlpm.g(_xlpm.g, 5))</f>
-        <v>120</v>
+        <f t="array" ref="A22">SUM(_xlfn.LAMBDA(_xlpm.a, _xlpm.a * 2)(F2:F5))</f>
+        <v>200</v>
       </c>
       <c r="B22">
-        <v>120</v>
+        <v>200</v>
       </c>
       <c r="C22" s="2" t="b">
-        <f t="shared" si="1"/>
+        <f>A22=B22</f>
         <v>1</v>
       </c>
       <c r="D22" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
-        <v>=LET(g, LAMBDA(self,n, IF(n &lt;= 1, 1, n * self(self, n - 1))), g(g, 5))</v>
+        <f ca="1">_xlfn.FORMULATEXT(A22)</f>
+        <v>=SUM(LAMBDA(a, a * 2)(F2:F5))</v>
       </c>
       <c r="E22" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" cm="1">
-        <f t="array" ref="A23">PLUS2(5)</f>
+        <f t="array" ref="A23">SUM(_xlfn.LAMBDA(_xlpm.a, _xlpm.a * 2)(DATARANGE))</f>
+        <v>200</v>
+      </c>
+      <c r="B23">
+        <v>200</v>
+      </c>
+      <c r="C23" s="2" t="b">
+        <f>A23=B23</f>
+        <v>1</v>
+      </c>
+      <c r="D23" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A23)</f>
+        <v>=SUM(LAMBDA(a, a * 2)(DATARANGE))</v>
+      </c>
+      <c r="E23" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" cm="1">
+        <f t="array" ref="A24">_xlfn.LET(_xlpm.g, _xlfn.LAMBDA(_xlpm.self,_xlpm.n, IF(_xlpm.n &lt;= 1, 1, _xlpm.n * _xlpm.self(_xlpm.self, _xlpm.n - 1))), _xlpm.g(_xlpm.g, 5))</f>
+        <v>120</v>
+      </c>
+      <c r="B24">
+        <v>120</v>
+      </c>
+      <c r="C24" s="2" t="b">
+        <f>A24=B24</f>
+        <v>1</v>
+      </c>
+      <c r="D24" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A24)</f>
+        <v>=LET(g, LAMBDA(self,n, IF(n &lt;= 1, 1, n * self(self, n - 1))), g(g, 5))</v>
+      </c>
+      <c r="E24" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" cm="1">
+        <f t="array" ref="A25">PLUS2(5)</f>
         <v>7</v>
       </c>
-      <c r="B23">
+      <c r="B25">
         <v>7</v>
       </c>
-      <c r="C23" s="2" t="b">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="D23" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="C25" s="2" t="b">
+        <f>A25=B25</f>
+        <v>1</v>
+      </c>
+      <c r="D25" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A25)</f>
         <v>=PLUS2(5)</v>
       </c>
-      <c r="E23" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5">
-      <c r="A24">
+      <c r="E25" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26">
         <f>SUM(4)</f>
         <v>4</v>
       </c>
-      <c r="B24">
+      <c r="B26">
         <v>4</v>
       </c>
-      <c r="C24" s="2" t="b">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="D24" s="1" t="str">
-        <f t="shared" ca="1" si="0"/>
+      <c r="C26" s="2" t="b">
+        <f>A26=B26</f>
+        <v>1</v>
+      </c>
+      <c r="D26" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A26)</f>
         <v>=SUM(4)</v>
       </c>
-      <c r="E24" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="E26" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" cm="1">
+        <f t="array" ref="A27">_xlfn.LAMBDA(_xlpm.x, SUM(_xlpm.x))(100)</f>
+        <v>100</v>
+      </c>
+      <c r="B27">
+        <v>100</v>
+      </c>
+      <c r="C27" s="2" t="b">
+        <f>A27=B27</f>
+        <v>1</v>
+      </c>
+      <c r="D27" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A27)</f>
+        <v>=LAMBDA(x, SUM(x))(100)</v>
+      </c>
+      <c r="E27" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" cm="1">
+        <f t="array" ref="A28">_xlfn.LAMBDA(_xlpm.x,_xlpm.f, _xlpm.f(_xlpm.x))(100,SUM)</f>
+        <v>110</v>
+      </c>
+      <c r="B28">
+        <v>110</v>
+      </c>
+      <c r="C28" s="2" t="b">
+        <f>A28=B28</f>
+        <v>1</v>
+      </c>
+      <c r="D28" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A28)</f>
+        <v>=LAMBDA(x,f, f(x))(100,SUM)</v>
+      </c>
+      <c r="E28" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" cm="1">
+        <f t="array" ref="A29">_xlfn.LAMBDA(_xlpm.f,_xlpm.n, _xlpm.f(_xlpm.n))(PLUS2, 1)</f>
+        <v>3</v>
+      </c>
+      <c r="B29">
+        <v>3</v>
+      </c>
+      <c r="C29" s="2" t="b">
+        <f>A29=B29</f>
+        <v>1</v>
+      </c>
+      <c r="D29" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A29)</f>
+        <v>=LAMBDA(f,n, f(n))(PLUS2, 1)</v>
+      </c>
+      <c r="E29" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" cm="1">
+        <f t="array" ref="A30">_xlfn.LAMBDA(_xlpm.f,_xlpm.n, _xlpm.f(_xlpm.n))(_xleta.COUNT, {1,2,3,4})</f>
+        <v>4</v>
+      </c>
+      <c r="B30">
+        <v>4</v>
+      </c>
+      <c r="C30" s="2" t="b">
+        <f>A30=B30</f>
+        <v>1</v>
+      </c>
+      <c r="D30" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A30)</f>
+        <v>=LAMBDA(f,n, f(n))(COUNT, {1,2,3,4})</v>
+      </c>
+      <c r="E30" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" cm="1">
+        <f t="array" ref="A31">_xlfn.LAMBDA(_xlpm.f, _xlpm.f(5))(_xlfn.LAMBDA(_xlpm.x, _xlpm.x * 2))</f>
+        <v>10</v>
+      </c>
+      <c r="B31">
+        <v>10</v>
+      </c>
+      <c r="C31" s="2" t="b">
+        <f>A31=B31</f>
+        <v>1</v>
+      </c>
+      <c r="D31" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A31)</f>
+        <v>=LAMBDA(f, f(5))(LAMBDA(x, x * 2))</v>
+      </c>
+      <c r="E31" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" cm="1">
+        <f t="array" ref="A32">_xlfn.LAMBDA(_xlpm.f,_xlpm.x, _xlpm.f(_xlpm.f(_xlpm.x)))(_xlfn.LAMBDA(_xlpm.n, _xlpm.n + 1), 5)</f>
+        <v>7</v>
+      </c>
+      <c r="B32">
+        <v>7</v>
+      </c>
+      <c r="C32" s="2" t="b">
+        <f>A32=B32</f>
+        <v>1</v>
+      </c>
+      <c r="D32" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A32)</f>
+        <v>=LAMBDA(f,x, f(f(x)))(LAMBDA(n, n + 1), 5)</v>
+      </c>
+      <c r="E32" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33" cm="1">
+        <f t="array" ref="A33">APPLYTWICE(_xlfn.LAMBDA(_xlpm.x, _xlpm.x * 2), 8)</f>
+        <v>32</v>
+      </c>
+      <c r="B33">
+        <v>32</v>
+      </c>
+      <c r="C33" s="2" t="b">
+        <f>A33=B33</f>
+        <v>1</v>
+      </c>
+      <c r="D33" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A33)</f>
+        <v>=APPLYTWICE(LAMBDA(x, x * 2), 8)</v>
+      </c>
+      <c r="E33" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34" cm="1">
+        <f t="array" ref="A34">_xlfn.LAMBDA(_xlpm.x, _xlpm.x + $F$2)(5)</f>
+        <v>15</v>
+      </c>
+      <c r="B34">
+        <v>15</v>
+      </c>
+      <c r="C34" s="2" t="b">
+        <f>A34=B34</f>
+        <v>1</v>
+      </c>
+      <c r="D34" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A34)</f>
+        <v>=LAMBDA(x, x + $F$2)(5)</v>
+      </c>
+      <c r="E34" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35" cm="1">
+        <f t="array" ref="A35">_xlfn.LAMBDA(_xlpm.a, _xlfn.LAMBDA(_xlpm.b, _xlfn.LAMBDA(_xlpm.c, _xlpm.a + _xlpm.b + _xlpm.c)))(3)(30)(300)</f>
+        <v>333</v>
+      </c>
+      <c r="B35">
+        <v>333</v>
+      </c>
+      <c r="C35" s="2" t="b">
+        <f>A35=B35</f>
+        <v>1</v>
+      </c>
+      <c r="D35" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A35)</f>
+        <v>=LAMBDA(a, LAMBDA(b, LAMBDA(c, a + b + c)))(3)(30)(300)</v>
+      </c>
+      <c r="E35" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5">
+      <c r="A36" cm="1">
+        <f t="array" ref="A36">_xlfn.LAMBDA(_xlpm.x,_xlpm.y, _xlpm.x + _xlpm.y)(20,)</f>
+        <v>20</v>
+      </c>
+      <c r="B36">
+        <v>20</v>
+      </c>
+      <c r="C36" s="2" t="b">
+        <f>A36=B36</f>
+        <v>1</v>
+      </c>
+      <c r="D36" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A36)</f>
+        <v>=LAMBDA(x,y, x + y)(20,)</v>
+      </c>
+      <c r="E36" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
+      <c r="A37" cm="1">
+        <f t="array" ref="A37">_xlfn.LAMBDA(_xlpm.x,_xlpm.y, _xlpm.x + _xlpm.y)(,2)</f>
+        <v>2</v>
+      </c>
+      <c r="B37">
+        <v>2</v>
+      </c>
+      <c r="C37" s="2" t="b">
+        <f>A37=B37</f>
+        <v>1</v>
+      </c>
+      <c r="D37" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A37)</f>
+        <v>=LAMBDA(x,y, x + y)(,2)</v>
+      </c>
+      <c r="E37" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5">
+      <c r="A38" cm="1">
+        <f t="array" ref="A38">_xlfn.LAMBDA(_xlpm.x,_xlop.y,_xlop.z, _xlpm.x + _xlpm.y + _xlpm.z)(7)</f>
+        <v>7</v>
+      </c>
+      <c r="B38">
+        <v>7</v>
+      </c>
+      <c r="C38" s="2" t="b">
+        <f>A38=B38</f>
+        <v>1</v>
+      </c>
+      <c r="D38" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A38)</f>
+        <v>=LAMBDA(x,[y],[z], x + y + z)(7)</v>
+      </c>
+      <c r="E38" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5">
+      <c r="A39" t="str" cm="1">
+        <f t="array" ref="A39">_xlfn.LAMBDA(_xlpm.x,_xlop.y,_xlop.z, _xlpm.x &amp; _xlpm.y &amp; _xlpm.z)("xy")</f>
+        <v>xy</v>
+      </c>
+      <c r="B39" t="s">
+        <v>44</v>
+      </c>
+      <c r="C39" s="2" t="b">
+        <f>A39=B39</f>
+        <v>1</v>
+      </c>
+      <c r="D39" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A39)</f>
+        <v>=LAMBDA(x,[y],[z], x &amp; y &amp; z)("xy")</v>
+      </c>
+      <c r="E39" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5">
+      <c r="A40" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C40" s="3"/>
+      <c r="D40" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E40" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5">
+      <c r="A41" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E41" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5">
+      <c r="A42" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5">
+      <c r="A43" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5">
+      <c r="A44" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B44" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5">
+      <c r="A45" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5">
+      <c r="A46" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5">
+      <c r="A47" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E47" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5">
+      <c r="A48" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1">
+      <c r="A49" s="3"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="C2:C39">
+    <cfRule type="cellIs" dxfId="7" priority="1" operator="notEqual">
+      <formula>TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5526BC4-8690-4B4D-B9FF-1C0DCDF78CF0}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="31.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="61.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="32.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="A1" s="4" t="s">
         <v>13</v>
       </c>
@@ -1238,7 +1940,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:6">
       <c r="A2" t="b" cm="1">
         <f t="array" ref="A2">_xlfn.LAMBDA(_xlpm.x,_xlpm.y, _xlfn.ISOMITTED(_xlpm.x))(, 5)</f>
         <v>1</v>
@@ -1247,7 +1949,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="b">
-        <f t="shared" ref="C2:C6" si="0">A2=B2</f>
+        <f t="shared" ref="C2:C11" si="0">A2=B2</f>
         <v>1</v>
       </c>
       <c r="D2" s="1" t="str">
@@ -1255,7 +1957,7 @@
         <v>=LAMBDA(x,y, ISOMITTED(x))(, 5)</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:6">
       <c r="A3" t="b" cm="1">
         <f t="array" ref="A3">_xlfn.LAMBDA(_xlpm.x,_xlpm.y, _xlfn.ISOMITTED(_xlpm.x))(3, 5)</f>
         <v>0</v>
@@ -1268,11 +1970,11 @@
         <v>1</v>
       </c>
       <c r="D3" s="1" t="str">
-        <f t="shared" ref="D3:D6" ca="1" si="1">_xlfn.FORMULATEXT(A3)</f>
+        <f t="shared" ref="D3:D8" ca="1" si="1">_xlfn.FORMULATEXT(A3)</f>
         <v>=LAMBDA(x,y, ISOMITTED(x))(3, 5)</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:6">
       <c r="A4" t="b" cm="1">
         <f t="array" ref="A4">_xlfn.LAMBDA(_xlpm.x,_xlpm.y, _xlfn.ISOMITTED(_xlpm.x))(3, 5)</f>
         <v>0</v>
@@ -1289,7 +1991,7 @@
         <v>=LAMBDA(x,y, ISOMITTED(x))(3, 5)</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:6">
       <c r="A5" cm="1">
         <f t="array" ref="A5">_xlfn.LAMBDA(_xlpm.x,_xlpm.y, IF(_xlfn.ISOMITTED(_xlpm.x), 99, _xlpm.x) + _xlpm.y)(, 5)</f>
         <v>104</v>
@@ -1306,7 +2008,7 @@
         <v>=LAMBDA(x,y, IF(ISOMITTED(x), 99, x) + y)(, 5)</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:6">
       <c r="A6" cm="1">
         <f t="array" ref="A6">_xlfn.LAMBDA(_xlpm.x,_xlpm.y, IF(_xlfn.ISOMITTED(_xlpm.x), 99, _xlpm.x) + _xlpm.y)(3, 5)</f>
         <v>8</v>
@@ -1323,24 +2025,131 @@
         <v>=LAMBDA(x,y, IF(ISOMITTED(x), 99, x) + y)(3, 5)</v>
       </c>
     </row>
+    <row r="7" spans="1:6">
+      <c r="A7">
+        <f>ERROR.TYPE(F7)</f>
+        <v>3</v>
+      </c>
+      <c r="B7">
+        <v>3</v>
+      </c>
+      <c r="C7" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="D7" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(F7)</f>
+        <v>=LAMBDA(x,y, ISOMITTED(y))(5)</v>
+      </c>
+      <c r="F7" t="e" cm="1" vm="1">
+        <f t="array" ref="F7">_xlfn.LAMBDA(_xlpm.x,_xlpm.y, _xlfn.ISOMITTED(_xlpm.y))(5)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" cm="1">
+        <f t="array" ref="A8">_xlfn.LAMBDA(_xlpm.a,_xlpm.b,_xlpm.c, IF(_xlfn.ISOMITTED(_xlpm.b), -1, _xlpm.b))(1, , 3)</f>
+        <v>-1</v>
+      </c>
+      <c r="B8">
+        <v>-1</v>
+      </c>
+      <c r="C8" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="D8" s="1" t="str">
+        <f t="shared" ca="1" si="1"/>
+        <v>=LAMBDA(a,b,c, IF(ISOMITTED(b), -1, b))(1, , 3)</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="3" cm="1">
+        <f t="array" ref="A9">_xlfn.LAMBDA(_xlop.x, IF(_xlfn.ISOMITTED(_xlpm.x),12,5))(1)</f>
+        <v>5</v>
+      </c>
+      <c r="B9">
+        <v>5</v>
+      </c>
+      <c r="C9" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="D9" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A9)</f>
+        <v>=LAMBDA([x], IF(ISOMITTED(x),12,5))(1)</v>
+      </c>
+      <c r="E9" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" cm="1">
+        <f t="array" ref="A10">_xlfn.LAMBDA(_xlop.x, IF(_xlfn.ISOMITTED(_xlpm.x),12,5))()</f>
+        <v>12</v>
+      </c>
+      <c r="B10">
+        <v>12</v>
+      </c>
+      <c r="C10" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="D10" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A10)</f>
+        <v>=LAMBDA([x], IF(ISOMITTED(x),12,5))()</v>
+      </c>
+      <c r="E10" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11">
+        <f>ERROR.TYPE(F11)</f>
+        <v>3</v>
+      </c>
+      <c r="B11">
+        <v>3</v>
+      </c>
+      <c r="C11" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="D11" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(F11)</f>
+        <v>=LAMBDA(x, IF(ISOMITTED(x),12,5))()</v>
+      </c>
+      <c r="E11" t="s">
+        <v>62</v>
+      </c>
+      <c r="F11" t="e" cm="1" vm="2">
+        <f t="array" ref="F11">_xlfn.LAMBDA(_xlpm.x, IF(_xlfn.ISOMITTED(_xlpm.x),12,5))()</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="C2:C11">
+    <cfRule type="cellIs" dxfId="6" priority="1" operator="notEqual">
+      <formula>TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39F3AAD1-330B-4374-B680-19CC9EB335F7}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.140625" customWidth="1"/>
     <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="86" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:8">
       <c r="A1" s="4" t="s">
         <v>13</v>
       </c>
@@ -1356,8 +2165,11 @@
       <c r="E1" s="4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="F1" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2">
         <f>SUM(_xlfn.BYCOL({1,2,3;4,5,6}, _xlfn.LAMBDA(_xlpm.c, SUM(_xlpm.c))))</f>
         <v>21</v>
@@ -1366,15 +2178,24 @@
         <v>21</v>
       </c>
       <c r="C2" t="b">
-        <f t="shared" ref="C2:C11" si="0">A2=B2</f>
+        <f t="shared" ref="C2:C14" si="0">A2=B2</f>
         <v>1</v>
       </c>
       <c r="D2" s="1" t="str">
         <f ca="1">_xlfn.FORMULATEXT(A2)</f>
         <v>=SUM(BYCOL({1,2,3;4,5,6}, LAMBDA(c, SUM(c))))</v>
       </c>
-    </row>
-    <row r="3" spans="1:5">
+      <c r="F2">
+        <v>11</v>
+      </c>
+      <c r="G2">
+        <v>22</v>
+      </c>
+      <c r="H2">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" cm="1">
         <f t="array" ref="A3">_xlfn.BYCOL({1;2;3}, _xlfn.LAMBDA(_xlpm.c, SUM(_xlpm.c)))</f>
         <v>6</v>
@@ -1387,11 +2208,20 @@
         <v>1</v>
       </c>
       <c r="D3" s="1" t="str">
-        <f t="shared" ref="D3:D10" ca="1" si="1">_xlfn.FORMULATEXT(A3)</f>
+        <f t="shared" ref="D3:D9" ca="1" si="1">_xlfn.FORMULATEXT(A3)</f>
         <v>=BYCOL({1;2;3}, LAMBDA(c, SUM(c)))</v>
       </c>
-    </row>
-    <row r="4" spans="1:5">
+      <c r="F3">
+        <v>44</v>
+      </c>
+      <c r="G3">
+        <v>55</v>
+      </c>
+      <c r="H3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4" cm="1">
         <f t="array" ref="A4:A6">TRANSPOSE(_xlfn.BYCOL({1,2,3;10,20,30}, _xlfn.LAMBDA(_xlpm.c, SUM(_xlpm.c))))</f>
         <v>11</v>
@@ -1407,8 +2237,17 @@
         <f t="shared" ca="1" si="1"/>
         <v>=TRANSPOSE(BYCOL({1,2,3;10,20,30}, LAMBDA(c, SUM(c))))</v>
       </c>
-    </row>
-    <row r="5" spans="1:5">
+      <c r="F4">
+        <v>77</v>
+      </c>
+      <c r="G4">
+        <v>88</v>
+      </c>
+      <c r="H4">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5">
         <v>22</v>
       </c>
@@ -1421,7 +2260,7 @@
       </c>
       <c r="D5" s="1"/>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:8">
       <c r="A6">
         <v>33</v>
       </c>
@@ -1434,7 +2273,7 @@
       </c>
       <c r="D6" s="1"/>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:8">
       <c r="A7" cm="1">
         <f t="array" ref="A7">_xlfn.BYCOL(100, _xlfn.LAMBDA(_xlpm.c, SUM(_xlpm.c)))</f>
         <v>100</v>
@@ -1451,13 +2290,13 @@
         <v>=BYCOL(100, LAMBDA(c, SUM(c)))</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:8">
       <c r="A8" t="str" cm="1">
         <f t="array" ref="A8">_xlfn.BYCOL("ABC", _xlfn.LAMBDA(_xlpm.c, _xlpm.c))</f>
         <v>ABC</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>63</v>
       </c>
       <c r="C8" t="b">
         <f t="shared" si="0"/>
@@ -1468,13 +2307,13 @@
         <v>=BYCOL("ABC", LAMBDA(c, c))</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:8">
       <c r="A9" s="3" t="str" cm="1">
         <f t="array" ref="A9:A11">TRANSPOSE(_xlfn.BYCOL({"A","B","C";"D","E","F"}, _xlfn.LAMBDA(_xlpm.c, _xlfn.CONCAT(_xlpm.c))))</f>
         <v>AD</v>
       </c>
       <c r="B9" t="s">
-        <v>23</v>
+        <v>64</v>
       </c>
       <c r="C9" t="b">
         <f t="shared" si="0"/>
@@ -1485,12 +2324,12 @@
         <v>=TRANSPOSE(BYCOL({"A","B","C";"D","E","F"}, LAMBDA(c, CONCAT(c))))</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:8">
       <c r="A10" t="str">
         <v>BE</v>
       </c>
       <c r="B10" t="s">
-        <v>24</v>
+        <v>65</v>
       </c>
       <c r="C10" t="b">
         <f t="shared" si="0"/>
@@ -1498,12 +2337,12 @@
       </c>
       <c r="D10" s="1"/>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:8">
       <c r="A11" t="str">
         <v>CF</v>
       </c>
       <c r="B11" t="s">
-        <v>25</v>
+        <v>66</v>
       </c>
       <c r="C11" t="b">
         <f t="shared" si="0"/>
@@ -1511,24 +2350,85 @@
       </c>
       <c r="D11" s="6"/>
     </row>
+    <row r="12" spans="1:8">
+      <c r="A12">
+        <f>F12</f>
+        <v>132</v>
+      </c>
+      <c r="B12">
+        <v>132</v>
+      </c>
+      <c r="C12" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="D12" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(F12)</f>
+        <v>=BYCOL(F2:H4, LAMBDA(c, SUM(c)))</v>
+      </c>
+      <c r="E12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F12" cm="1">
+        <f t="array" ref="F12:H12">_xlfn.BYCOL(F2:H4, _xlfn.LAMBDA(_xlpm.c, SUM(_xlpm.c)))</f>
+        <v>132</v>
+      </c>
+      <c r="G12">
+        <v>165</v>
+      </c>
+      <c r="H12">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13">
+        <f>G12</f>
+        <v>165</v>
+      </c>
+      <c r="B13">
+        <v>165</v>
+      </c>
+      <c r="C13" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14">
+        <f>H12</f>
+        <v>198</v>
+      </c>
+      <c r="B14">
+        <v>198</v>
+      </c>
+      <c r="C14" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="C2:C14">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="notEqual">
+      <formula>TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EE8A135-F1D7-4292-81A0-1877087BD36C}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.5703125" customWidth="1"/>
     <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="71.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="32" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:8">
       <c r="A1" s="4" t="s">
         <v>13</v>
       </c>
@@ -1544,8 +2444,11 @@
       <c r="E1" s="4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="F1" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2">
         <f>SUM(_xlfn.BYROW({1,2,3;4,5,6}, _xlfn.LAMBDA(_xlpm.c, SUM(_xlpm.c))))</f>
         <v>21</v>
@@ -1554,15 +2457,24 @@
         <v>21</v>
       </c>
       <c r="C2" t="b">
-        <f t="shared" ref="C2:C9" si="0">A2=B2</f>
+        <f t="shared" ref="C2:C14" si="0">A2=B2</f>
         <v>1</v>
       </c>
       <c r="D2" s="1" t="str">
         <f ca="1">_xlfn.FORMULATEXT(A2)</f>
         <v>=SUM(BYROW({1,2,3;4,5,6}, LAMBDA(c, SUM(c))))</v>
       </c>
-    </row>
-    <row r="3" spans="1:5">
+      <c r="F2">
+        <v>11</v>
+      </c>
+      <c r="G2">
+        <v>22</v>
+      </c>
+      <c r="H2">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" cm="1">
         <f t="array" ref="A3">_xlfn.BYROW({1,2,3}, _xlfn.LAMBDA(_xlpm.c, SUM(_xlpm.c)))</f>
         <v>6</v>
@@ -1578,8 +2490,17 @@
         <f t="shared" ref="D3:D9" ca="1" si="1">_xlfn.FORMULATEXT(A3)</f>
         <v>=BYROW({1,2,3}, LAMBDA(c, SUM(c)))</v>
       </c>
-    </row>
-    <row r="4" spans="1:5">
+      <c r="F3">
+        <v>44</v>
+      </c>
+      <c r="G3">
+        <v>55</v>
+      </c>
+      <c r="H3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4" cm="1">
         <f t="array" ref="A4:A5">_xlfn.BYROW({1,2,3;10,20,30}, _xlfn.LAMBDA(_xlpm.c, SUM(_xlpm.c)))</f>
         <v>6</v>
@@ -1595,8 +2516,17 @@
         <f t="shared" ca="1" si="1"/>
         <v>=BYROW({1,2,3;10,20,30}, LAMBDA(c, SUM(c)))</v>
       </c>
-    </row>
-    <row r="5" spans="1:5">
+      <c r="F4">
+        <v>77</v>
+      </c>
+      <c r="G4">
+        <v>88</v>
+      </c>
+      <c r="H4">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5">
         <v>60</v>
       </c>
@@ -1609,7 +2539,7 @@
       </c>
       <c r="D5" s="1"/>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:8">
       <c r="A6" cm="1">
         <f t="array" ref="A6">_xlfn.BYROW(100, _xlfn.LAMBDA(_xlpm.c, SUM(_xlpm.c)))</f>
         <v>100</v>
@@ -1626,13 +2556,13 @@
         <v>=BYROW(100, LAMBDA(c, SUM(c)))</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:8">
       <c r="A7" t="str" cm="1">
         <f t="array" ref="A7">_xlfn.BYROW("ABC", _xlfn.LAMBDA(_xlpm.c, _xlpm.c))</f>
         <v>ABC</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
+        <v>63</v>
       </c>
       <c r="C7" t="b">
         <f t="shared" si="0"/>
@@ -1643,13 +2573,13 @@
         <v>=BYROW("ABC", LAMBDA(c, c))</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:8">
       <c r="A8" s="3" t="str" cm="1">
         <f t="array" ref="A8:A9">_xlfn.BYROW({"A","B","C";"D","E","F"}, _xlfn.LAMBDA(_xlpm.c, _xlfn.CONCAT(_xlpm.c)))</f>
         <v>ABC</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>63</v>
       </c>
       <c r="C8" t="b">
         <f t="shared" si="0"/>
@@ -1660,12 +2590,12 @@
         <v>=BYROW({"A","B","C";"D","E","F"}, LAMBDA(c, CONCAT(c)))</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:8">
       <c r="A9" t="str">
         <v>DEF</v>
       </c>
       <c r="B9" t="s">
-        <v>26</v>
+        <v>68</v>
       </c>
       <c r="C9" t="b">
         <f t="shared" si="0"/>
@@ -1673,14 +2603,92 @@
       </c>
       <c r="D9" s="1"/>
     </row>
+    <row r="10" spans="1:8">
+      <c r="A10" cm="1">
+        <f t="array" ref="A10:A12">_xlfn.BYROW(F2:H4, _xlfn.LAMBDA(_xlpm.c, SUM(_xlpm.c)))</f>
+        <v>66</v>
+      </c>
+      <c r="B10">
+        <v>66</v>
+      </c>
+      <c r="C10" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="D10" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A10)</f>
+        <v>=BYROW(F2:H4, LAMBDA(c, SUM(c)))</v>
+      </c>
+      <c r="E10" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11">
+        <v>165</v>
+      </c>
+      <c r="B11">
+        <v>165</v>
+      </c>
+      <c r="C11" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12">
+        <v>264</v>
+      </c>
+      <c r="B12">
+        <v>264</v>
+      </c>
+      <c r="C12" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" cm="1">
+        <f t="array" ref="A13:A14">_xlfn.BYROW({1,2;3,4}, _xlfn.LAMBDA(_xlpm.r, _xlfn.REDUCE(0, _xlpm.r, _xlfn.LAMBDA(_xlpm.a,_xlpm.v, _xlpm.a + _xlpm.v))))</f>
+        <v>3</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="D13" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A13)</f>
+        <v>=BYROW({1,2;3,4}, LAMBDA(r, REDUCE(0, r, LAMBDA(a,v, a + v))))</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14">
+        <v>7</v>
+      </c>
+      <c r="B14">
+        <v>7</v>
+      </c>
+      <c r="C14" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="C2:C14">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="notEqual">
+      <formula>TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5A7ED71-DF37-4E12-B0D5-80D8154AC7BB}">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1707,7 +2715,7 @@
         <v>17</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>27</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -1834,40 +2842,107 @@
       </c>
     </row>
     <row r="9" spans="1:7">
-      <c r="A9" t="e" cm="1">
-        <f t="array" ref="A9">_xlfn.MAKEARRAY(0, 3, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, 1))</f>
+      <c r="A9">
+        <f>ERROR.TYPE(F9)</f>
+        <v>3</v>
+      </c>
+      <c r="B9">
+        <v>3</v>
+      </c>
+      <c r="C9" t="b">
+        <f>A9=B9</f>
+        <v>1</v>
+      </c>
+      <c r="D9" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(F9)</f>
+        <v>=MAKEARRAY(0, 3, LAMBDA(r,c, 1))</v>
+      </c>
+      <c r="F9" t="e" cm="1">
+        <f t="array" ref="F9">_xlfn.MAKEARRAY(0, 3, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, 1))</f>
         <v>#VALUE!</v>
       </c>
-      <c r="B9" t="e">
-        <v>#VALUE!</v>
-      </c>
-      <c r="C9" t="b">
-        <f>IF(ERROR.TYPE(A9) = 3, TRUE, FALSE)</f>
-        <v>1</v>
-      </c>
-      <c r="D9" s="1" t="str">
-        <f ca="1">_xlfn.FORMULATEXT(A9)</f>
-        <v>=MAKEARRAY(0, 3, LAMBDA(r,c, 1))</v>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" cm="1">
+        <f t="array" ref="A10:A11">_xlfn.MAKEARRAY(2, 1, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, _xlpm.r + _xlpm.c))</f>
+        <v>2</v>
+      </c>
+      <c r="B10">
+        <v>2</v>
+      </c>
+      <c r="C10" t="b">
+        <f>A10=B10</f>
+        <v>1</v>
+      </c>
+      <c r="D10" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A10)</f>
+        <v>=MAKEARRAY(2, 1, LAMBDA(r,c, r + c))</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11">
+        <v>3</v>
+      </c>
+      <c r="B11">
+        <v>3</v>
+      </c>
+      <c r="C11" t="b">
+        <f>A11=B11</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" cm="1">
+        <f t="array" ref="A12:A13">_xlfn.MAKEARRAY(2, 1, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, 6))</f>
+        <v>6</v>
+      </c>
+      <c r="B12">
+        <v>6</v>
+      </c>
+      <c r="C12" t="b">
+        <f>A12=B12</f>
+        <v>1</v>
+      </c>
+      <c r="D12" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A12)</f>
+        <v>=MAKEARRAY(2, 1, LAMBDA(r,c, 6))</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13">
+        <v>6</v>
+      </c>
+      <c r="B13">
+        <v>6</v>
+      </c>
+      <c r="C13" t="b">
+        <f>A13=B13</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="C2:C13">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="notEqual">
+      <formula>TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37D895F7-4E9F-442E-ADEB-EE55261ADDAB}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="73.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="A1" s="4" t="s">
         <v>13</v>
       </c>
@@ -1883,10 +2958,13 @@
       <c r="E1" s="4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="F1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2" cm="1">
-        <f t="array" ref="A2:A4">TRANSPOSE(_xlfn.MAP({1,2,3}, _xlfn.LAMBDA(_xlpm.x, _xlpm.x * _xlpm.x)))</f>
+        <f t="array" ref="A2:A4">_xlfn.MAP({1;2;3}, _xlfn.LAMBDA(_xlpm.x, _xlpm.x * _xlpm.x))</f>
         <v>1</v>
       </c>
       <c r="B2">
@@ -1898,10 +2976,13 @@
       </c>
       <c r="D2" s="7" t="str">
         <f ca="1">_xlfn.FORMULATEXT(A2)</f>
-        <v>=TRANSPOSE(MAP({1,2,3}, LAMBDA(x, x * x)))</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
+        <v>=MAP({1;2;3}, LAMBDA(x, x * x))</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3">
         <v>4</v>
       </c>
@@ -1913,8 +2994,11 @@
         <v>1</v>
       </c>
       <c r="D3" s="7"/>
-    </row>
-    <row r="4" spans="1:5">
+      <c r="F3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4">
         <v>9</v>
       </c>
@@ -1926,10 +3010,13 @@
         <v>1</v>
       </c>
       <c r="D4" s="7"/>
-    </row>
-    <row r="5" spans="1:5">
+      <c r="F4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5" cm="1">
-        <f t="array" ref="A5:A7">TRANSPOSE(_xlfn.MAP({1,2,3}, {10,20,30}, _xlfn.LAMBDA(_xlpm.a,_xlpm.b, _xlpm.a + _xlpm.b)))</f>
+        <f t="array" ref="A5:A7">_xlfn.MAP({1;2;3}, {10;20;30}, _xlfn.LAMBDA(_xlpm.a,_xlpm.b, _xlpm.a + _xlpm.b))</f>
         <v>11</v>
       </c>
       <c r="B5">
@@ -1941,10 +3028,13 @@
       </c>
       <c r="D5" s="7" t="str">
         <f ca="1">_xlfn.FORMULATEXT(A5)</f>
-        <v>=TRANSPOSE(MAP({1,2,3}, {10,20,30}, LAMBDA(a,b, a + b)))</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
+        <v>=MAP({1;2;3}, {10;20;30}, LAMBDA(a,b, a + b))</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
       <c r="A6">
         <v>22</v>
       </c>
@@ -1957,7 +3047,7 @@
       </c>
       <c r="D6" s="7"/>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:6">
       <c r="A7">
         <v>33</v>
       </c>
@@ -1970,13 +3060,13 @@
       </c>
       <c r="D7" s="7"/>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:6">
       <c r="A8" t="str" cm="1">
-        <f t="array" ref="A8:A9">TRANSPOSE(_xlfn.MAP({"a","b"}, _xlfn.LAMBDA(_xlpm.x, UPPER(_xlpm.x))))</f>
+        <f t="array" ref="A8:A9">_xlfn.MAP({"a";"b"}, _xlfn.LAMBDA(_xlpm.x, UPPER(_xlpm.x)))</f>
         <v>A</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>71</v>
       </c>
       <c r="C8" t="b">
         <f>A8=B8</f>
@@ -1984,15 +3074,15 @@
       </c>
       <c r="D8" s="7" t="str">
         <f ca="1">_xlfn.FORMULATEXT(A8)</f>
-        <v>=TRANSPOSE(MAP({"a","b"}, LAMBDA(x, UPPER(x))))</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
+        <v>=MAP({"a";"b"}, LAMBDA(x, UPPER(x)))</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9" t="str">
         <v>B</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
+        <v>72</v>
       </c>
       <c r="C9" t="b">
         <f>A9=B9</f>
@@ -2000,24 +3090,198 @@
       </c>
       <c r="D9" s="7"/>
     </row>
+    <row r="10" spans="1:6">
+      <c r="A10" cm="1">
+        <f t="array" ref="A10:A13">_xlfn.MAP(F2:F5, _xlfn.LAMBDA(_xlpm.x, _xlpm.x * _xlpm.x))</f>
+        <v>4</v>
+      </c>
+      <c r="B10">
+        <v>4</v>
+      </c>
+      <c r="C10" t="b">
+        <f t="shared" ref="C10:C20" si="0">A10=B10</f>
+        <v>1</v>
+      </c>
+      <c r="D10" s="7" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A10)</f>
+        <v>=MAP(F2:F5, LAMBDA(x, x * x))</v>
+      </c>
+      <c r="E10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11">
+        <v>25</v>
+      </c>
+      <c r="B11">
+        <v>25</v>
+      </c>
+      <c r="C11" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12">
+        <v>4</v>
+      </c>
+      <c r="B12">
+        <v>4</v>
+      </c>
+      <c r="C12" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13">
+        <v>1</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="D13" s="7"/>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" cm="1">
+        <f t="array" ref="A14:A16">_xlfn.LET(_xlpm.double, _xlfn.LAMBDA(_xlpm.x, _xlpm.x * 2), _xlfn.MAP({1;2;3}, _xlpm.double))</f>
+        <v>2</v>
+      </c>
+      <c r="B14">
+        <v>2</v>
+      </c>
+      <c r="C14" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="D14" s="7" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A14)</f>
+        <v>=LET(double, LAMBDA(x, x * 2), MAP({1;2;3}, double))</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15">
+        <v>4</v>
+      </c>
+      <c r="B15">
+        <v>4</v>
+      </c>
+      <c r="C15" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16">
+        <v>6</v>
+      </c>
+      <c r="B16">
+        <v>6</v>
+      </c>
+      <c r="C16" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" cm="1">
+        <f t="array" ref="A17">SUM(IFERROR(_xlfn.MAP({1,0,2}, _xlfn.LAMBDA(_xlpm.x, 1 / _xlpm.x)), 0))</f>
+        <v>1.5</v>
+      </c>
+      <c r="B17">
+        <v>1.5</v>
+      </c>
+      <c r="C17" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="D17" s="7" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A17)</f>
+        <v>=SUM(IFERROR(MAP({1,0,2}, LAMBDA(x, 1 / x)), 0))</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18">
+        <f>F18</f>
+        <v>2</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="D18" s="7" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(F18)</f>
+        <v>=MAP({1;2;3}, {1;2}, LAMBDA(a,b, a + b))</v>
+      </c>
+      <c r="F18" cm="1">
+        <f t="array" ref="F18:F20">_xlfn.MAP({1;2;3}, {1;2}, _xlfn.LAMBDA(_xlpm.a,_xlpm.b, _xlpm.a + _xlpm.b))</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19">
+        <f>F19</f>
+        <v>4</v>
+      </c>
+      <c r="B19">
+        <v>4</v>
+      </c>
+      <c r="C19" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="F19">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20">
+        <f>ERROR.TYPE(F20)</f>
+        <v>7</v>
+      </c>
+      <c r="B20">
+        <v>7</v>
+      </c>
+      <c r="C20" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="D20" s="7"/>
+      <c r="F20" t="e">
+        <v>#N/A</v>
+      </c>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="C2:C20">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="notEqual">
+      <formula>TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB2CDB70-0194-415F-9EDC-5C927CB1F6B2}">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="70.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="78.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:7">
       <c r="A1" s="4" t="s">
         <v>13</v>
       </c>
@@ -2033,8 +3297,14 @@
       <c r="E1" s="4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="F1" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2" cm="1">
         <f t="array" ref="A2">_xlfn.REDUCE(0, {1,2,3,4}, _xlfn.LAMBDA(_xlpm.acc,_xlpm.val, _xlpm.acc + _xlpm.val))</f>
         <v>10</v>
@@ -2050,8 +3320,14 @@
         <f ca="1">_xlfn.FORMULATEXT(A2)</f>
         <v>=REDUCE(0, {1,2,3,4}, LAMBDA(acc,val, acc + val))</v>
       </c>
-    </row>
-    <row r="3" spans="1:5">
+      <c r="F2">
+        <v>12</v>
+      </c>
+      <c r="G2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
       <c r="A3" cm="1">
         <f t="array" ref="A3">_xlfn.REDUCE(1, {1,2,3,4}, _xlfn.LAMBDA(_xlpm.acc,_xlpm.val, _xlpm.acc * _xlpm.val))</f>
         <v>24</v>
@@ -2064,17 +3340,23 @@
         <v>1</v>
       </c>
       <c r="D3" s="1" t="str">
-        <f t="shared" ref="D3:D5" ca="1" si="0">_xlfn.FORMULATEXT(A3)</f>
+        <f t="shared" ref="D3:D7" ca="1" si="0">_xlfn.FORMULATEXT(A3)</f>
         <v>=REDUCE(1, {1,2,3,4}, LAMBDA(acc,val, acc * val))</v>
       </c>
-    </row>
-    <row r="4" spans="1:5">
+      <c r="F3">
+        <v>14</v>
+      </c>
+      <c r="G3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
       <c r="A4" t="str" cm="1">
         <f t="array" ref="A4">_xlfn.REDUCE("", {"a","b","c"}, _xlfn.LAMBDA(_xlpm.acc,_xlpm.val, _xlpm.acc &amp; _xlpm.val))</f>
         <v>abc</v>
       </c>
       <c r="B4" t="s">
-        <v>30</v>
+        <v>76</v>
       </c>
       <c r="C4" t="b">
         <f>A4=B4</f>
@@ -2084,14 +3366,20 @@
         <f t="shared" ca="1" si="0"/>
         <v>=REDUCE("", {"a","b","c"}, LAMBDA(acc,val, acc &amp; val))</v>
       </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" cm="1">
-        <f t="array" ref="A5">_xlfn.REDUCE(, {1,2,3}, _xlfn.LAMBDA(_xlpm.acc,_xlpm.val, _xlpm.acc + _xlpm.val))</f>
-        <v>6</v>
-      </c>
-      <c r="B5">
-        <v>6</v>
+      <c r="F4">
+        <v>11</v>
+      </c>
+      <c r="G4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="str" cm="1">
+        <f t="array" ref="A5">_xlfn.REDUCE(10 &amp; "_", {"a","b","c"}, _xlfn.LAMBDA(_xlpm.acc,_xlpm.val, _xlpm.acc &amp; _xlpm.val))</f>
+        <v>10_abc</v>
+      </c>
+      <c r="B5" t="s">
+        <v>77</v>
       </c>
       <c r="C5" t="b">
         <f>A5=B5</f>
@@ -2099,17 +3387,116 @@
       </c>
       <c r="D5" s="1" t="str">
         <f t="shared" ca="1" si="0"/>
+        <v>=REDUCE(10 &amp; "_", {"a","b","c"}, LAMBDA(acc,val, acc &amp; val))</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" cm="1">
+        <f t="array" ref="A6">_xlfn.REDUCE(, {1,2,3}, _xlfn.LAMBDA(_xlpm.acc,_xlpm.val, _xlpm.acc + _xlpm.val))</f>
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>6</v>
+      </c>
+      <c r="C6" t="b">
+        <f>A6=B6</f>
+        <v>1</v>
+      </c>
+      <c r="D6" s="1" t="str">
+        <f t="shared" ca="1" si="0"/>
         <v>=REDUCE(, {1,2,3}, LAMBDA(acc,val, acc + val))</v>
       </c>
     </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="3" cm="1">
+        <f t="array" ref="A7">_xlfn.REDUCE(5, {1,2,3;4,5,6}, _xlfn.LAMBDA(_xlpm.acc,_xlpm.val, _xlpm.acc + _xlpm.val))</f>
+        <v>26</v>
+      </c>
+      <c r="B7">
+        <v>26</v>
+      </c>
+      <c r="C7" t="b">
+        <f>A7=B7</f>
+        <v>1</v>
+      </c>
+      <c r="D7" s="1" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>=REDUCE(5, {1,2,3;4,5,6}, LAMBDA(acc,val, acc + val))</v>
+      </c>
+      <c r="E7" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" cm="1">
+        <f t="array" ref="A8">_xlfn.REDUCE(2, F2:F4, _xlfn.LAMBDA(_xlpm.acc,_xlpm.val, _xlpm.acc + _xlpm.val))</f>
+        <v>39</v>
+      </c>
+      <c r="B8">
+        <v>39</v>
+      </c>
+      <c r="C8" t="b">
+        <f>A8=B8</f>
+        <v>1</v>
+      </c>
+      <c r="D8" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A8)</f>
+        <v>=REDUCE(2, F2:F4, LAMBDA(acc,val, acc + val))</v>
+      </c>
+      <c r="E8" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" cm="1">
+        <f t="array" ref="A9">_xlfn.REDUCE(10, _xlfn.UNIQUE(G2:G4), _xlfn.LAMBDA(_xlpm.acc,_xlpm.val, _xlpm.acc + _xlpm.val))</f>
+        <v>18</v>
+      </c>
+      <c r="B9">
+        <v>18</v>
+      </c>
+      <c r="C9" t="b">
+        <f>A9=B9</f>
+        <v>1</v>
+      </c>
+      <c r="D9" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A9)</f>
+        <v>=REDUCE(10, UNIQUE(G2:G4), LAMBDA(acc,val, acc + val))</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="3" cm="1">
+        <f t="array" ref="A10">IFERROR(_xlfn.REDUCE(0, {1,0}, _xlfn.LAMBDA(_xlpm.acc,_xlpm.val, _xlpm.acc / _xlpm.val)), -1)</f>
+        <v>-1</v>
+      </c>
+      <c r="B10">
+        <v>-1</v>
+      </c>
+      <c r="C10" t="b">
+        <f>A10=B10</f>
+        <v>1</v>
+      </c>
+      <c r="D10" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(A10)</f>
+        <v>=IFERROR(REDUCE(0, {1,0}, LAMBDA(acc,val, acc / val)), -1)</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="D11" s="1"/>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="C2:C10">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="notEqual">
+      <formula>TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FD896EE-D870-48CB-919F-FA13DBBB7395}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -2205,7 +3592,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="7" t="str">
-        <f t="shared" ref="D3:D8" ca="1" si="0">_xlfn.FORMULATEXT(A6)</f>
+        <f t="shared" ref="D3:D9" ca="1" si="0">_xlfn.FORMULATEXT(A6)</f>
         <v>=TRANSPOSE(SCAN(, {1,2,3}, LAMBDA(acc,val, acc + val)))</v>
       </c>
     </row>
@@ -2235,7 +3622,53 @@
       </c>
       <c r="D8" s="7"/>
     </row>
+    <row r="9" spans="1:5">
+      <c r="A9" t="str" cm="1">
+        <f t="array" ref="A9:A11">_xlfn.SCAN("a", {"a";"b";"c"}, _xlfn.LAMBDA(_xlpm.acc,_xlpm.val, _xlpm.acc &amp; _xlpm.val))</f>
+        <v>aa</v>
+      </c>
+      <c r="B9" t="s">
+        <v>80</v>
+      </c>
+      <c r="C9" t="b">
+        <f>A9=B9</f>
+        <v>1</v>
+      </c>
+      <c r="D9" s="7" t="str">
+        <f t="shared" ca="1" si="0"/>
+        <v>=SCAN("a", {"a";"b";"c"}, LAMBDA(acc,val, acc &amp; val))</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" t="str">
+        <v>aab</v>
+      </c>
+      <c r="B10" t="s">
+        <v>81</v>
+      </c>
+      <c r="C10" t="b">
+        <f>A10=B10</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" t="str">
+        <v>aabc</v>
+      </c>
+      <c r="B11" t="s">
+        <v>82</v>
+      </c>
+      <c r="C11" t="b">
+        <f>A11=B11</f>
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="C2:C11">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="notEqual">
+      <formula>TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>